<commit_message>
Add CalcMethod and StatsFinding sheets to ASR_Paper_Data.xlsx
- CalcMethod: step-by-step extraction logic for word count, speaker count,
  and total markers (regex patterns per notation with explanations), plus
  raw data matrices (5 models × 4 clips) with mean/SD/CV per notation
- StatsFinding: CV analysis identifying Total Markers as the primary
  discriminating metric (CV 0.41–0.61); model ranking by notation richness

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ASR_Paper_Data.xlsx
+++ b/data/ASR_Paper_Data.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Muller_Models" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelSummary" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FileIndex" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CalcMethod" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StatsFinding" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="68">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -186,8 +188,178 @@
       <color rgb="00888888"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffffff"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffffff"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00333333"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000d47a1"/>
+    </font>
+    <font>
+      <color rgb="00444444"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffffff"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00222222"/>
+    </font>
+    <font>
+      <color rgb="000d47a1"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00999999"/>
+    </font>
+    <font>
+      <color rgb="00333333"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00222222"/>
+    </font>
+    <font>
+      <color rgb="00cc0000"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0081C784"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0022543d"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="00a8d8a8"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <color rgb="00333333"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00444444"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00ffffff"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004FC3F7"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00222222"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <color rgb="00444444"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFB74D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CE93D8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000d47a1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0081C784"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00aaaaaa"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00222222"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="000d47a1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00006600"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00cc0000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00cc6600"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
@@ -214,8 +386,143 @@
         <fgColor rgb="000a0a18"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000d0d2a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a1a3a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e0e4ee"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f0f4ff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff0f0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff8f0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f8f8f8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e3f2fd"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8f5e9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff8e1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f3e5f5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fce4ec"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e0f7fa"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001e3a5f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f0fff4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000d1117"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f8fff8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f5f5ff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002a2a4a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fafafa"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8f4fd"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f5faff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000d2a1a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8e8ff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff3e0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f9f9f9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a3a2a"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -223,11 +530,83 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00cccccc"/>
+      </left>
+      <right style="thin">
+        <color rgb="00cccccc"/>
+      </right>
+      <top style="thin">
+        <color rgb="00cccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00cccccc"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00cccccc"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00cccccc"/>
+      </right>
+      <top style="thin">
+        <color rgb="00cccccc"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00cccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00cccccc"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00cccccc"/>
+      </right>
+      <top style="thin">
+        <color rgb="00cccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00cccccc"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00dddddd"/>
+      </left>
+      <right style="thin">
+        <color rgb="00dddddd"/>
+      </right>
+      <top style="thin">
+        <color rgb="00dddddd"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00dddddd"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -407,6 +786,317 @@
     <xf numFmtId="0" fontId="19" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="26" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="27" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="29" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="61" fillId="29" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="30" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="29" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="31" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1157,6 +1847,627 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="69" t="inlineStr">
+        <is>
+          <t>STATS FINDING — Most Impactful Metrics for Model Comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="70" t="inlineStr">
+        <is>
+          <t>Generated 2026-06-04  ·  5 models × 4 notations × 4 clips (N=80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="71" t="inlineStr">
+        <is>
+          <t>KEY FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="72" t="inlineStr">
+        <is>
+          <t>★ Primary metric</t>
+        </is>
+      </c>
+      <c r="B5" s="73" t="inlineStr">
+        <is>
+          <t>Total Markers</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="inlineStr">
+        <is>
+          <t>CV 0.41–0.61 across notations — highest between-model variance. Recommended as the lead quantitative metric in the paper.</t>
+        </is>
+      </c>
+      <c r="D5" s="174" t="n"/>
+      <c r="E5" s="174" t="n"/>
+      <c r="F5" s="174" t="n"/>
+      <c r="G5" s="174" t="n"/>
+      <c r="H5" s="174" t="n"/>
+      <c r="I5" s="174" t="n"/>
+      <c r="J5" s="174" t="n"/>
+      <c r="K5" s="175" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>✗ Weakest metric</t>
+        </is>
+      </c>
+      <c r="B6" s="77" t="inlineStr">
+        <is>
+          <t>Word Count</t>
+        </is>
+      </c>
+      <c r="C6" s="78" t="inlineStr">
+        <is>
+          <t>CV 0.06–0.10 — minimal variation across models. All models produce similar word counts; not useful for between-model comparison.</t>
+        </is>
+      </c>
+      <c r="D6" s="174" t="n"/>
+      <c r="E6" s="174" t="n"/>
+      <c r="F6" s="174" t="n"/>
+      <c r="G6" s="174" t="n"/>
+      <c r="H6" s="174" t="n"/>
+      <c r="I6" s="174" t="n"/>
+      <c r="J6" s="174" t="n"/>
+      <c r="K6" s="175" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>⚠ Secondary metric</t>
+        </is>
+      </c>
+      <c r="B7" s="80" t="inlineStr">
+        <is>
+          <t>Speakers detected</t>
+        </is>
+      </c>
+      <c r="C7" s="81" t="inlineStr">
+        <is>
+          <t>CV 0.42–0.91 — varies but noisy. Gemini Flash outlier (mean 4.6, max 14). Use with caution; may reflect prompt behaviour not acoustic reality.</t>
+        </is>
+      </c>
+      <c r="D7" s="174" t="n"/>
+      <c r="E7" s="174" t="n"/>
+      <c r="F7" s="174" t="n"/>
+      <c r="G7" s="174" t="n"/>
+      <c r="H7" s="174" t="n"/>
+      <c r="I7" s="174" t="n"/>
+      <c r="J7" s="174" t="n"/>
+      <c r="K7" s="175" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="72" t="inlineStr">
+        <is>
+          <t>★ Best notation for discrimination</t>
+        </is>
+      </c>
+      <c r="B8" s="73" t="inlineStr">
+        <is>
+          <t>Müller &amp; Guendouzi (2005)</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>CV=0.61, range=50 markers. Largest spread between models — strongest notation for demonstrating model differences in the paper.</t>
+        </is>
+      </c>
+      <c r="D8" s="174" t="n"/>
+      <c r="E8" s="174" t="n"/>
+      <c r="F8" s="174" t="n"/>
+      <c r="G8" s="174" t="n"/>
+      <c r="H8" s="174" t="n"/>
+      <c r="I8" s="174" t="n"/>
+      <c r="J8" s="174" t="n"/>
+      <c r="K8" s="175" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>↓ Lowest notation discrimination</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr">
+        <is>
+          <t>Braun &amp; Clarke (2021)</t>
+        </is>
+      </c>
+      <c r="C9" s="84" t="inlineStr">
+        <is>
+          <t>CV=0.41, range=12. Simpler system; models converge more. Still useful as contrast to Jefferson/Müller.</t>
+        </is>
+      </c>
+      <c r="D9" s="174" t="n"/>
+      <c r="E9" s="174" t="n"/>
+      <c r="F9" s="174" t="n"/>
+      <c r="G9" s="174" t="n"/>
+      <c r="H9" s="174" t="n"/>
+      <c r="I9" s="174" t="n"/>
+      <c r="J9" s="174" t="n"/>
+      <c r="K9" s="175" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>↑ Highest-performing model</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr">
+        <is>
+          <t>GPT-audio</t>
+        </is>
+      </c>
+      <c r="C10" s="84" t="inlineStr">
+        <is>
+          <t>Most notation-rich overall (avg 62.5 markers in Müller). Applies widest range of markers.</t>
+        </is>
+      </c>
+      <c r="D10" s="174" t="n"/>
+      <c r="E10" s="174" t="n"/>
+      <c r="F10" s="174" t="n"/>
+      <c r="G10" s="174" t="n"/>
+      <c r="H10" s="174" t="n"/>
+      <c r="I10" s="174" t="n"/>
+      <c r="J10" s="174" t="n"/>
+      <c r="K10" s="175" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>↓ Lowest-performing model</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr">
+        <is>
+          <t>GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="C11" s="84" t="inlineStr">
+        <is>
+          <t>Consistently fewest markers across all notations (1.75–12.5). 3–13× fewer than top models.</t>
+        </is>
+      </c>
+      <c r="D11" s="174" t="n"/>
+      <c r="E11" s="174" t="n"/>
+      <c r="F11" s="174" t="n"/>
+      <c r="G11" s="174" t="n"/>
+      <c r="H11" s="174" t="n"/>
+      <c r="I11" s="174" t="n"/>
+      <c r="J11" s="174" t="n"/>
+      <c r="K11" s="175" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>DISCRIMINATING POWER — Coefficient of Variation (CV = SD/Mean) per Notation × Metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="85" t="inlineStr">
+        <is>
+          <t>Notation</t>
+        </is>
+      </c>
+      <c r="B14" s="85" t="inlineStr">
+        <is>
+          <t>TotalMrk
+CV</t>
+        </is>
+      </c>
+      <c r="C14" s="85" t="inlineStr">
+        <is>
+          <t>TotalMrk
+Range</t>
+        </is>
+      </c>
+      <c r="D14" s="85" t="inlineStr">
+        <is>
+          <t>TotalMrk
+Max/Min×</t>
+        </is>
+      </c>
+      <c r="E14" s="85" t="inlineStr">
+        <is>
+          <t>WordCnt
+CV</t>
+        </is>
+      </c>
+      <c r="F14" s="85" t="inlineStr">
+        <is>
+          <t>WordCnt
+Range</t>
+        </is>
+      </c>
+      <c r="G14" s="85" t="inlineStr">
+        <is>
+          <t>WordCnt
+Max/Min×</t>
+        </is>
+      </c>
+      <c r="H14" s="85" t="inlineStr">
+        <is>
+          <t>Speakers
+CV</t>
+        </is>
+      </c>
+      <c r="I14" s="85" t="inlineStr">
+        <is>
+          <t>Speakers
+Range</t>
+        </is>
+      </c>
+      <c r="J14" s="85" t="inlineStr">
+        <is>
+          <t>Speakers
+Max/Min×</t>
+        </is>
+      </c>
+      <c r="K14" s="85" t="inlineStr">
+        <is>
+          <t>Recommended
+Metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="86" t="inlineStr">
+        <is>
+          <t>Jefferson (CA)</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C15" s="88" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="D15" s="88" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="E15" s="89" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="89" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G15" s="89" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H15" s="88" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I15" s="88" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J15" s="88" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K15" s="90" t="inlineStr">
+        <is>
+          <t>Total Markers (CV=0.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="91" t="inlineStr">
+        <is>
+          <t>Poland (2001)</t>
+        </is>
+      </c>
+      <c r="B16" s="92" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C16" s="93" t="n">
+        <v>26</v>
+      </c>
+      <c r="D16" s="93" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="94" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F16" s="94" t="n">
+        <v>29</v>
+      </c>
+      <c r="G16" s="94" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H16" s="93" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I16" s="93" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J16" s="93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="95" t="inlineStr">
+        <is>
+          <t>Total Markers (CV=0.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="96" t="inlineStr">
+        <is>
+          <t>Braun &amp; Clarke (2021)</t>
+        </is>
+      </c>
+      <c r="B17" s="97" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C17" s="98" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D17" s="98" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E17" s="99" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F17" s="99" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="G17" s="99" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H17" s="98" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="I17" s="98" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="98" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" s="100" t="inlineStr">
+        <is>
+          <t>Total Markers (CV=0.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="101" t="inlineStr">
+        <is>
+          <t>Müller &amp; Guendouzi (2005)</t>
+        </is>
+      </c>
+      <c r="B18" s="102" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="C18" s="103" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="103" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="104" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F18" s="104" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G18" s="104" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H18" s="103" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I18" s="103" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J18" s="103" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K18" s="105" t="inlineStr">
+        <is>
+          <t>Total Markers (CV=0.61) ★</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="71" t="inlineStr">
+        <is>
+          <t>MODEL RANKING — Avg Total Markers per Notation (across 4 clips)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="85" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B21" s="85" t="inlineStr">
+        <is>
+          <t>Jefferson
+(CA)</t>
+        </is>
+      </c>
+      <c r="C21" s="85" t="inlineStr">
+        <is>
+          <t>Poland
+(2001)</t>
+        </is>
+      </c>
+      <c r="D21" s="85" t="inlineStr">
+        <is>
+          <t>Braun &amp;
+Clarke</t>
+        </is>
+      </c>
+      <c r="E21" s="85" t="inlineStr">
+        <is>
+          <t>Müller
+(2005)</t>
+        </is>
+      </c>
+      <c r="F21" s="85" t="inlineStr">
+        <is>
+          <t>Avg all
+notations</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="91" t="inlineStr">
+        <is>
+          <t>1. GPT-audio</t>
+        </is>
+      </c>
+      <c r="B22" s="106" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C22" s="106" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="D22" s="106" t="n">
+        <v>17</v>
+      </c>
+      <c r="E22" s="106" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="F22" s="107" t="n">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="108" t="inlineStr">
+        <is>
+          <t>2. Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="B23" s="88" t="n">
+        <v>23</v>
+      </c>
+      <c r="C23" s="88" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D23" s="88" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E23" s="88" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F23" s="109" t="n">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="110" t="inlineStr">
+        <is>
+          <t>3. WhisperX medium</t>
+        </is>
+      </c>
+      <c r="B24" s="111" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C24" s="111" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" s="111" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E24" s="111" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="F24" s="112" t="n">
+        <v>20.1</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="113" t="inlineStr">
+        <is>
+          <t>4. Gemini 2.5 Flash</t>
+        </is>
+      </c>
+      <c r="B25" s="114" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C25" s="114" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D25" s="114" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E25" s="114" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F25" s="115" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="116" t="inlineStr">
+        <is>
+          <t>5. GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="B26" s="98" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C26" s="98" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D26" s="98" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E26" s="98" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F26" s="117" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="C11:K11"/>
+    <mergeCell ref="C10:K10"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="C9:K9"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="C8:K8"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="C6:K6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -12977,4 +14288,2929 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0034A853"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I127"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="69" t="inlineStr">
+        <is>
+          <t>CALCULATION METHOD — How Metrics Are Extracted from Transcript .txt Files</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="118" t="inlineStr">
+        <is>
+          <t>Source: generate_paper_data.py  ·  All metrics computed from indexed .txt transcript files  ·  80 files (5 models × 4 notations × 4 clips)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="119" t="inlineStr">
+        <is>
+          <t>STEP 1 — Locate the Correct .txt File (find_transcript)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="120" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B5" s="120" t="inlineStr">
+        <is>
+          <t>Pattern / value</t>
+        </is>
+      </c>
+      <c r="C5" s="121" t="n"/>
+      <c r="D5" s="121" t="n"/>
+      <c r="E5" s="120" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+      <c r="F5" s="121" t="n"/>
+      <c r="G5" s="121" t="n"/>
+      <c r="H5" s="121" t="n"/>
+      <c r="I5" s="121" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="122" t="inlineStr">
+        <is>
+          <t>Naming pattern</t>
+        </is>
+      </c>
+      <c r="B6" s="123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {clip_stem}_{Model}_{Notation}_Indexed_{timestamp}.txt</t>
+        </is>
+      </c>
+      <c r="C6" s="121" t="n"/>
+      <c r="D6" s="121" t="n"/>
+      <c r="E6" s="124" t="inlineStr">
+        <is>
+          <t>Each file encodes clip, model, and notation in its name. The script uses glob() to find the most recent file for each combination.</t>
+        </is>
+      </c>
+      <c r="F6" s="121" t="n"/>
+      <c r="G6" s="121" t="n"/>
+      <c r="H6" s="121" t="n"/>
+      <c r="I6" s="121" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="122" t="inlineStr">
+        <is>
+          <t>WhisperX path</t>
+        </is>
+      </c>
+      <c r="B7" s="123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  outputs/{stem}_WhisperX/{stem}_WhisperX_{Notation}_Indexed_*.txt</t>
+        </is>
+      </c>
+      <c r="C7" s="121" t="n"/>
+      <c r="D7" s="121" t="n"/>
+      <c r="E7" s="124" t="inlineStr">
+        <is>
+          <t>2-step pipeline: WhisperX ASR runs first and saves its output in a subdirectory. The LLM then applies notation to that text.</t>
+        </is>
+      </c>
+      <c r="F7" s="121" t="n"/>
+      <c r="G7" s="121" t="n"/>
+      <c r="H7" s="121" t="n"/>
+      <c r="I7" s="121" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="122" t="inlineStr">
+        <is>
+          <t>Müller path</t>
+        </is>
+      </c>
+      <c r="B8" s="123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  outputs/Muller_Notation/{stem}_{Model}_Muller_Indexed_*.txt</t>
+        </is>
+      </c>
+      <c r="C8" s="121" t="n"/>
+      <c r="D8" s="121" t="n"/>
+      <c r="E8" s="124" t="inlineStr">
+        <is>
+          <t>Müller notation was generated separately (run_muller_notation.sh) and lives in its own folder.</t>
+        </is>
+      </c>
+      <c r="F8" s="121" t="n"/>
+      <c r="G8" s="121" t="n"/>
+      <c r="H8" s="121" t="n"/>
+      <c r="I8" s="121" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="122" t="inlineStr">
+        <is>
+          <t>Missing file</t>
+        </is>
+      </c>
+      <c r="B9" s="123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  all metrics = 0, Found = "–"</t>
+        </is>
+      </c>
+      <c r="C9" s="121" t="n"/>
+      <c r="D9" s="121" t="n"/>
+      <c r="E9" s="124" t="inlineStr">
+        <is>
+          <t>Logged in the FileIndex sheet. Means either the LLM generation failed or the file has not been generated yet.</t>
+        </is>
+      </c>
+      <c r="F9" s="121" t="n"/>
+      <c r="G9" s="121" t="n"/>
+      <c r="H9" s="121" t="n"/>
+      <c r="I9" s="121" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="119" t="inlineStr">
+        <is>
+          <t>STEP 2 — Word Count  (_word_count function)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="120" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B12" s="120" t="inlineStr">
+        <is>
+          <t>Python code</t>
+        </is>
+      </c>
+      <c r="C12" s="121" t="n"/>
+      <c r="D12" s="121" t="n"/>
+      <c r="E12" s="120" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+      <c r="F12" s="121" t="n"/>
+      <c r="G12" s="121" t="n"/>
+      <c r="H12" s="121" t="n"/>
+      <c r="I12" s="121" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="122" t="inlineStr">
+        <is>
+          <t>Strip ## header</t>
+        </is>
+      </c>
+      <c r="B13" s="123" t="inlineStr">
+        <is>
+          <t>re.sub(r"##.*", "", text)</t>
+        </is>
+      </c>
+      <c r="C13" s="121" t="n"/>
+      <c r="D13" s="121" t="n"/>
+      <c r="E13" s="124" t="inlineStr">
+        <is>
+          <t>Removes the "## Model Transcript — filename" line at the top of every indexed file.</t>
+        </is>
+      </c>
+      <c r="F13" s="121" t="n"/>
+      <c r="G13" s="121" t="n"/>
+      <c r="H13" s="121" t="n"/>
+      <c r="I13" s="121" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="122" t="inlineStr">
+        <is>
+          <t>Remove (( )) tags</t>
+        </is>
+      </c>
+      <c r="B14" s="123" t="inlineStr">
+        <is>
+          <t>re.sub(r"\(\(.*?\)\)", " ", text)</t>
+        </is>
+      </c>
+      <c r="C14" s="121" t="n"/>
+      <c r="D14" s="121" t="n"/>
+      <c r="E14" s="124" t="inlineStr">
+        <is>
+          <t>Replaces non-verbal annotations like ((laughs)) with a space — these are transcriber comments, not spoken words.</t>
+        </is>
+      </c>
+      <c r="F14" s="121" t="n"/>
+      <c r="G14" s="121" t="n"/>
+      <c r="H14" s="121" t="n"/>
+      <c r="I14" s="121" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="122" t="inlineStr">
+        <is>
+          <t>Count word tokens</t>
+        </is>
+      </c>
+      <c r="B15" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\b\w+\b", clean))</t>
+        </is>
+      </c>
+      <c r="C15" s="121" t="n"/>
+      <c r="D15" s="121" t="n"/>
+      <c r="E15" s="124" t="inlineStr">
+        <is>
+          <t>\b\w+\b matches sequences of letters/digits at word boundaries. Notation symbols (brackets, arrows, colons) are excluded because \w only matches [A-Za-z0-9_].</t>
+        </is>
+      </c>
+      <c r="F15" s="121" t="n"/>
+      <c r="G15" s="121" t="n"/>
+      <c r="H15" s="121" t="n"/>
+      <c r="I15" s="121" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="119" t="inlineStr">
+        <is>
+          <t>STEP 3 — Speaker Count  (_unique_speakers function)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="120" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B18" s="120" t="inlineStr">
+        <is>
+          <t>Code / Pattern</t>
+        </is>
+      </c>
+      <c r="C18" s="121" t="n"/>
+      <c r="D18" s="121" t="n"/>
+      <c r="E18" s="120" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F18" s="121" t="n"/>
+      <c r="G18" s="121" t="n"/>
+      <c r="H18" s="121" t="n"/>
+      <c r="I18" s="121" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="122" t="inlineStr">
+        <is>
+          <t>Generic label pattern</t>
+        </is>
+      </c>
+      <c r="B19" s="123" t="inlineStr">
+        <is>
+          <t>Speaker [A-Z]:</t>
+        </is>
+      </c>
+      <c r="C19" s="121" t="n"/>
+      <c r="D19" s="121" t="n"/>
+      <c r="E19" s="124" t="inlineStr">
+        <is>
+          <t>Matches "Speaker A:", "Speaker B:", etc. — the standard format used in this study.</t>
+        </is>
+      </c>
+      <c r="F19" s="121" t="n"/>
+      <c r="G19" s="121" t="n"/>
+      <c r="H19" s="121" t="n"/>
+      <c r="I19" s="121" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="122" t="inlineStr">
+        <is>
+          <t>Named speaker pattern</t>
+        </is>
+      </c>
+      <c r="B20" s="123" t="inlineStr">
+        <is>
+          <t>[A-Z][a-z]+:</t>
+        </is>
+      </c>
+      <c r="C20" s="121" t="n"/>
+      <c r="D20" s="121" t="n"/>
+      <c r="E20" s="124" t="inlineStr">
+        <is>
+          <t>Matches character names like "Houston:" or "Jim:" when the model uses names instead of generic labels.</t>
+        </is>
+      </c>
+      <c r="F20" s="121" t="n"/>
+      <c r="G20" s="121" t="n"/>
+      <c r="H20" s="121" t="n"/>
+      <c r="I20" s="121" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="122" t="inlineStr">
+        <is>
+          <t>Deduplicate</t>
+        </is>
+      </c>
+      <c r="B21" s="123" t="inlineStr">
+        <is>
+          <t>set(re.findall(...))</t>
+        </is>
+      </c>
+      <c r="C21" s="121" t="n"/>
+      <c r="D21" s="121" t="n"/>
+      <c r="E21" s="124" t="inlineStr">
+        <is>
+          <t>Wraps findall in a set — each unique speaker label counted once regardless of turn count.</t>
+        </is>
+      </c>
+      <c r="F21" s="121" t="n"/>
+      <c r="G21" s="121" t="n"/>
+      <c r="H21" s="121" t="n"/>
+      <c r="I21" s="121" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="122" t="inlineStr">
+        <is>
+          <t>Return value</t>
+        </is>
+      </c>
+      <c r="B22" s="123" t="inlineStr">
+        <is>
+          <t>len(set)</t>
+        </is>
+      </c>
+      <c r="C22" s="121" t="n"/>
+      <c r="D22" s="121" t="n"/>
+      <c r="E22" s="124" t="inlineStr">
+        <is>
+          <t>Total unique speakers detected. This is a model behaviour metric; it may differ from the ground-truth speaker count.</t>
+        </is>
+      </c>
+      <c r="F22" s="121" t="n"/>
+      <c r="G22" s="121" t="n"/>
+      <c r="H22" s="121" t="n"/>
+      <c r="I22" s="121" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="119" t="inlineStr">
+        <is>
+          <t>STEP 4 — Total Markers  (notation-specific regex, sum of all sub-marker counts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="125" t="inlineStr">
+        <is>
+          <t>Each notation has a dedicated extractor function. Each function runs a set of regex patterns against the transcript text. Each match = 1 marker. Total Markers = sum of all sub-marker counts for that notation. A "marker" is any notation symbol the model inserted — brackets, arrows, pauses, emphasis marks, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Notation: Jefferson (CA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="127" t="inlineStr">
+        <is>
+          <t>Marker name</t>
+        </is>
+      </c>
+      <c r="B27" s="127" t="inlineStr">
+        <is>
+          <t>Python regex</t>
+        </is>
+      </c>
+      <c r="C27" s="121" t="n"/>
+      <c r="D27" s="121" t="n"/>
+      <c r="E27" s="127" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F27" s="121" t="n"/>
+      <c r="G27" s="121" t="n"/>
+      <c r="H27" s="121" t="n"/>
+      <c r="I27" s="121" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="128" t="inlineStr">
+        <is>
+          <t>Overlaps [</t>
+        </is>
+      </c>
+      <c r="B28" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\[", re.sub(r"\[\d{2}:\d{2}\]","",text)))</t>
+        </is>
+      </c>
+      <c r="C28" s="121" t="n"/>
+      <c r="D28" s="121" t="n"/>
+      <c r="E28" s="129" t="inlineStr">
+        <is>
+          <t>Strip timestamp brackets [00:15] first, then count remaining [ as overlap markers.</t>
+        </is>
+      </c>
+      <c r="F28" s="121" t="n"/>
+      <c r="G28" s="121" t="n"/>
+      <c r="H28" s="121" t="n"/>
+      <c r="I28" s="121" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="128" t="inlineStr">
+        <is>
+          <t>Latching =</t>
+        </is>
+      </c>
+      <c r="B29" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"=", text))</t>
+        </is>
+      </c>
+      <c r="C29" s="121" t="n"/>
+      <c r="D29" s="121" t="n"/>
+      <c r="E29" s="129" t="inlineStr">
+        <is>
+          <t>Counts = signs (latched/immediate continuation).</t>
+        </is>
+      </c>
+      <c r="F29" s="121" t="n"/>
+      <c r="G29" s="121" t="n"/>
+      <c r="H29" s="121" t="n"/>
+      <c r="I29" s="121" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="128" t="inlineStr">
+        <is>
+          <t>Micro pause (.)</t>
+        </is>
+      </c>
+      <c r="B30" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\.\)", text))</t>
+        </is>
+      </c>
+      <c r="C30" s="121" t="n"/>
+      <c r="D30" s="121" t="n"/>
+      <c r="E30" s="129" t="inlineStr">
+        <is>
+          <t>Literal string (.) — one-beat pause.</t>
+        </is>
+      </c>
+      <c r="F30" s="121" t="n"/>
+      <c r="G30" s="121" t="n"/>
+      <c r="H30" s="121" t="n"/>
+      <c r="I30" s="121" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="128" t="inlineStr">
+        <is>
+          <t>Timed pause (n.n)</t>
+        </is>
+      </c>
+      <c r="B31" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\d+\.\d+\)", text))</t>
+        </is>
+      </c>
+      <c r="C31" s="121" t="n"/>
+      <c r="D31" s="121" t="n"/>
+      <c r="E31" s="129" t="inlineStr">
+        <is>
+          <t>Decimal-number pauses like (1.2), (0.8).</t>
+        </is>
+      </c>
+      <c r="F31" s="121" t="n"/>
+      <c r="G31" s="121" t="n"/>
+      <c r="H31" s="121" t="n"/>
+      <c r="I31" s="121" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="128" t="inlineStr">
+        <is>
+          <t>Pitch up/down</t>
+        </is>
+      </c>
+      <c r="B32" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"[↑↓]", text))</t>
+        </is>
+      </c>
+      <c r="C32" s="121" t="n"/>
+      <c r="D32" s="121" t="n"/>
+      <c r="E32" s="129" t="inlineStr">
+        <is>
+          <t>Unicode pitch arrows counted together.</t>
+        </is>
+      </c>
+      <c r="F32" s="121" t="n"/>
+      <c r="G32" s="121" t="n"/>
+      <c r="H32" s="121" t="n"/>
+      <c r="I32" s="121" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="128" t="inlineStr">
+        <is>
+          <t>Lengthening ::</t>
+        </is>
+      </c>
+      <c r="B33" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r":{2,}", text))</t>
+        </is>
+      </c>
+      <c r="C33" s="121" t="n"/>
+      <c r="D33" s="121" t="n"/>
+      <c r="E33" s="129" t="inlineStr">
+        <is>
+          <t>2+ consecutive colons.</t>
+        </is>
+      </c>
+      <c r="F33" s="121" t="n"/>
+      <c r="G33" s="121" t="n"/>
+      <c r="H33" s="121" t="n"/>
+      <c r="I33" s="121" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="128" t="inlineStr">
+        <is>
+          <t>Breath .hhh</t>
+        </is>
+      </c>
+      <c r="B34" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\.hhh", text))</t>
+        </is>
+      </c>
+      <c r="C34" s="121" t="n"/>
+      <c r="D34" s="121" t="n"/>
+      <c r="E34" s="129" t="inlineStr">
+        <is>
+          <t>.hhh sequence (in-breath).</t>
+        </is>
+      </c>
+      <c r="F34" s="121" t="n"/>
+      <c r="G34" s="121" t="n"/>
+      <c r="H34" s="121" t="n"/>
+      <c r="I34" s="121" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="128" t="inlineStr">
+        <is>
+          <t>Emphasis _word_</t>
+        </is>
+      </c>
+      <c r="B35" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"_\w+_", text))</t>
+        </is>
+      </c>
+      <c r="C35" s="121" t="n"/>
+      <c r="D35" s="121" t="n"/>
+      <c r="E35" s="129" t="inlineStr">
+        <is>
+          <t>Underscore-wrapped word token (\w+ = letters/digits).</t>
+        </is>
+      </c>
+      <c r="F35" s="121" t="n"/>
+      <c r="G35" s="121" t="n"/>
+      <c r="H35" s="121" t="n"/>
+      <c r="I35" s="121" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="128" t="inlineStr">
+        <is>
+          <t>Rising ¿</t>
+        </is>
+      </c>
+      <c r="B36" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"¿", text))</t>
+        </is>
+      </c>
+      <c r="C36" s="121" t="n"/>
+      <c r="D36" s="121" t="n"/>
+      <c r="E36" s="129" t="inlineStr">
+        <is>
+          <t>Inverted question mark (weak rising) — ¿ not ? to avoid English punctuation collision.</t>
+        </is>
+      </c>
+      <c r="F36" s="121" t="n"/>
+      <c r="G36" s="121" t="n"/>
+      <c r="H36" s="121" t="n"/>
+      <c r="I36" s="121" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="128" t="inlineStr">
+        <is>
+          <t>Paralinguistic ((</t>
+        </is>
+      </c>
+      <c r="B37" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\(", text))</t>
+        </is>
+      </c>
+      <c r="C37" s="121" t="n"/>
+      <c r="D37" s="121" t="n"/>
+      <c r="E37" s="129" t="inlineStr">
+        <is>
+          <t>Double open-parenthesis for non-verbal annotations.</t>
+        </is>
+      </c>
+      <c r="F37" s="121" t="n"/>
+      <c r="G37" s="121" t="n"/>
+      <c r="H37" s="121" t="n"/>
+      <c r="I37" s="121" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="128" t="inlineStr">
+        <is>
+          <t>Marked →</t>
+        </is>
+      </c>
+      <c r="B38" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"→", text))</t>
+        </is>
+      </c>
+      <c r="C38" s="121" t="n"/>
+      <c r="D38" s="121" t="n"/>
+      <c r="E38" s="129" t="inlineStr">
+        <is>
+          <t>Rightward arrow (noticeably marked turn).</t>
+        </is>
+      </c>
+      <c r="F38" s="121" t="n"/>
+      <c r="G38" s="121" t="n"/>
+      <c r="H38" s="121" t="n"/>
+      <c r="I38" s="121" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Notation: Poland (2001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="120" t="inlineStr">
+        <is>
+          <t>Marker name</t>
+        </is>
+      </c>
+      <c r="B41" s="120" t="inlineStr">
+        <is>
+          <t>Python regex</t>
+        </is>
+      </c>
+      <c r="C41" s="121" t="n"/>
+      <c r="D41" s="121" t="n"/>
+      <c r="E41" s="120" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F41" s="121" t="n"/>
+      <c r="G41" s="121" t="n"/>
+      <c r="H41" s="121" t="n"/>
+      <c r="I41" s="121" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="130" t="inlineStr">
+        <is>
+          <t>Short pause ..</t>
+        </is>
+      </c>
+      <c r="B42" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"(?&lt;!\.)\.\.(?!\.)", text))</t>
+        </is>
+      </c>
+      <c r="C42" s="121" t="n"/>
+      <c r="D42" s="121" t="n"/>
+      <c r="E42" s="129" t="inlineStr">
+        <is>
+          <t>Exactly two dots using negative lookahead/lookbehind to exclude longer sequences like ...</t>
+        </is>
+      </c>
+      <c r="F42" s="121" t="n"/>
+      <c r="G42" s="121" t="n"/>
+      <c r="H42" s="121" t="n"/>
+      <c r="I42" s="121" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="130" t="inlineStr">
+        <is>
+          <t>Long pause ...</t>
+        </is>
+      </c>
+      <c r="B43" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\.{3,}", text))</t>
+        </is>
+      </c>
+      <c r="C43" s="121" t="n"/>
+      <c r="D43" s="121" t="n"/>
+      <c r="E43" s="129" t="inlineStr">
+        <is>
+          <t>3+ consecutive dots.</t>
+        </is>
+      </c>
+      <c r="F43" s="121" t="n"/>
+      <c r="G43" s="121" t="n"/>
+      <c r="H43" s="121" t="n"/>
+      <c r="I43" s="121" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="130" t="inlineStr">
+        <is>
+          <t>(overlapping)</t>
+        </is>
+      </c>
+      <c r="B44" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(overlapping\)", text, re.I))</t>
+        </is>
+      </c>
+      <c r="C44" s="121" t="n"/>
+      <c r="D44" s="121" t="n"/>
+      <c r="E44" s="129" t="inlineStr">
+        <is>
+          <t>Literal word (overlapping) in parentheses.</t>
+        </is>
+      </c>
+      <c r="F44" s="121" t="n"/>
+      <c r="G44" s="121" t="n"/>
+      <c r="H44" s="121" t="n"/>
+      <c r="I44" s="121" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="130" t="inlineStr">
+        <is>
+          <t>CAPS emphasis</t>
+        </is>
+      </c>
+      <c r="B45" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\b[A-Z]{2,}\b", text))</t>
+        </is>
+      </c>
+      <c r="C45" s="121" t="n"/>
+      <c r="D45" s="121" t="n"/>
+      <c r="E45" s="129" t="inlineStr">
+        <is>
+          <t>Sequences of 2+ capital letters as a word boundary.</t>
+        </is>
+      </c>
+      <c r="F45" s="121" t="n"/>
+      <c r="G45" s="121" t="n"/>
+      <c r="H45" s="121" t="n"/>
+      <c r="I45" s="121" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="130" t="inlineStr">
+        <is>
+          <t>Paralinguistic</t>
+        </is>
+      </c>
+      <c r="B46" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\((laughing|coughs|sigh|…)\)", text, re.I))</t>
+        </is>
+      </c>
+      <c r="C46" s="121" t="n"/>
+      <c r="D46" s="121" t="n"/>
+      <c r="E46" s="129" t="inlineStr">
+        <is>
+          <t>Named non-verbal behaviours in parentheses.</t>
+        </is>
+      </c>
+      <c r="F46" s="121" t="n"/>
+      <c r="G46" s="121" t="n"/>
+      <c r="H46" s="121" t="n"/>
+      <c r="I46" s="121" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="130" t="inlineStr">
+        <is>
+          <t>Inaudible xxxxx</t>
+        </is>
+      </c>
+      <c r="B47" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\bx{2,}\b", text, re.I))</t>
+        </is>
+      </c>
+      <c r="C47" s="121" t="n"/>
+      <c r="D47" s="121" t="n"/>
+      <c r="E47" s="129" t="inlineStr">
+        <is>
+          <t>2+ x characters as a word (inaudible speech).</t>
+        </is>
+      </c>
+      <c r="F47" s="121" t="n"/>
+      <c r="G47" s="121" t="n"/>
+      <c r="H47" s="121" t="n"/>
+      <c r="I47" s="121" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="130" t="inlineStr">
+        <is>
+          <t>Reported speech ""</t>
+        </is>
+      </c>
+      <c r="B48" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\"[^\"]{3,}\"", text))</t>
+        </is>
+      </c>
+      <c r="C48" s="121" t="n"/>
+      <c r="D48" s="121" t="n"/>
+      <c r="E48" s="129" t="inlineStr">
+        <is>
+          <t>Quoted strings of 3+ characters.</t>
+        </is>
+      </c>
+      <c r="F48" s="121" t="n"/>
+      <c r="G48" s="121" t="n"/>
+      <c r="H48" s="121" t="n"/>
+      <c r="I48" s="121" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Notation: Braun &amp; Clarke (2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="131" t="inlineStr">
+        <is>
+          <t>Marker name</t>
+        </is>
+      </c>
+      <c r="B51" s="131" t="inlineStr">
+        <is>
+          <t>Python regex</t>
+        </is>
+      </c>
+      <c r="C51" s="121" t="n"/>
+      <c r="D51" s="121" t="n"/>
+      <c r="E51" s="131" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F51" s="121" t="n"/>
+      <c r="G51" s="121" t="n"/>
+      <c r="H51" s="121" t="n"/>
+      <c r="I51" s="121" t="n"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="132" t="inlineStr">
+        <is>
+          <t>Micro pause (.)</t>
+        </is>
+      </c>
+      <c r="B52" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\.\)", text))</t>
+        </is>
+      </c>
+      <c r="C52" s="121" t="n"/>
+      <c r="D52" s="121" t="n"/>
+      <c r="E52" s="129" t="inlineStr">
+        <is>
+          <t>Single dot in parentheses.</t>
+        </is>
+      </c>
+      <c r="F52" s="121" t="n"/>
+      <c r="G52" s="121" t="n"/>
+      <c r="H52" s="121" t="n"/>
+      <c r="I52" s="121" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="132" t="inlineStr">
+        <is>
+          <t>Short pause (..)</t>
+        </is>
+      </c>
+      <c r="B53" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\.\.\)", text))</t>
+        </is>
+      </c>
+      <c r="C53" s="121" t="n"/>
+      <c r="D53" s="121" t="n"/>
+      <c r="E53" s="129" t="inlineStr">
+        <is>
+          <t>Two dots in parentheses.</t>
+        </is>
+      </c>
+      <c r="F53" s="121" t="n"/>
+      <c r="G53" s="121" t="n"/>
+      <c r="H53" s="121" t="n"/>
+      <c r="I53" s="121" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="132" t="inlineStr">
+        <is>
+          <t>Long pause (...)</t>
+        </is>
+      </c>
+      <c r="B54" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\.\.\.\)", text))</t>
+        </is>
+      </c>
+      <c r="C54" s="121" t="n"/>
+      <c r="D54" s="121" t="n"/>
+      <c r="E54" s="129" t="inlineStr">
+        <is>
+          <t>Three dots in parentheses.</t>
+        </is>
+      </c>
+      <c r="F54" s="121" t="n"/>
+      <c r="G54" s="121" t="n"/>
+      <c r="H54" s="121" t="n"/>
+      <c r="I54" s="121" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="132" t="inlineStr">
+        <is>
+          <t>Paralinguistic ((</t>
+        </is>
+      </c>
+      <c r="B55" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\(", text))</t>
+        </is>
+      </c>
+      <c r="C55" s="121" t="n"/>
+      <c r="D55" s="121" t="n"/>
+      <c r="E55" s="129" t="inlineStr">
+        <is>
+          <t>Double open-parenthesis.</t>
+        </is>
+      </c>
+      <c r="F55" s="121" t="n"/>
+      <c r="G55" s="121" t="n"/>
+      <c r="H55" s="121" t="n"/>
+      <c r="I55" s="121" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="132" t="inlineStr">
+        <is>
+          <t>[unclear]</t>
+        </is>
+      </c>
+      <c r="B56" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\[unclear\]", text, re.I))</t>
+        </is>
+      </c>
+      <c r="C56" s="121" t="n"/>
+      <c r="D56" s="121" t="n"/>
+      <c r="E56" s="129" t="inlineStr">
+        <is>
+          <t>Literal [unclear] tag.</t>
+        </is>
+      </c>
+      <c r="F56" s="121" t="n"/>
+      <c r="G56" s="121" t="n"/>
+      <c r="H56" s="121" t="n"/>
+      <c r="I56" s="121" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="132" t="inlineStr">
+        <is>
+          <t>[overlap]</t>
+        </is>
+      </c>
+      <c r="B57" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\[overlap\]", text, re.I))</t>
+        </is>
+      </c>
+      <c r="C57" s="121" t="n"/>
+      <c r="D57" s="121" t="n"/>
+      <c r="E57" s="129" t="inlineStr">
+        <is>
+          <t>Literal [overlap] tag.</t>
+        </is>
+      </c>
+      <c r="F57" s="121" t="n"/>
+      <c r="G57" s="121" t="n"/>
+      <c r="H57" s="121" t="n"/>
+      <c r="I57" s="121" t="n"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="132" t="inlineStr">
+        <is>
+          <t>Emphasis *word*</t>
+        </is>
+      </c>
+      <c r="B58" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\*\w+\*", text))</t>
+        </is>
+      </c>
+      <c r="C58" s="121" t="n"/>
+      <c r="D58" s="121" t="n"/>
+      <c r="E58" s="129" t="inlineStr">
+        <is>
+          <t>Asterisk-wrapped word (\w+).</t>
+        </is>
+      </c>
+      <c r="F58" s="121" t="n"/>
+      <c r="G58" s="121" t="n"/>
+      <c r="H58" s="121" t="n"/>
+      <c r="I58" s="121" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Notation: Müller &amp; Guendouzi (2005)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="133" t="inlineStr">
+        <is>
+          <t>Marker name</t>
+        </is>
+      </c>
+      <c r="B61" s="133" t="inlineStr">
+        <is>
+          <t>Python regex</t>
+        </is>
+      </c>
+      <c r="C61" s="121" t="n"/>
+      <c r="D61" s="121" t="n"/>
+      <c r="E61" s="133" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F61" s="121" t="n"/>
+      <c r="G61" s="121" t="n"/>
+      <c r="H61" s="121" t="n"/>
+      <c r="I61" s="121" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="134" t="inlineStr">
+        <is>
+          <t>Rising ¿</t>
+        </is>
+      </c>
+      <c r="B62" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"¿", text))</t>
+        </is>
+      </c>
+      <c r="C62" s="121" t="n"/>
+      <c r="D62" s="121" t="n"/>
+      <c r="E62" s="129" t="inlineStr">
+        <is>
+          <t>¿ replaces original ? — avoids collision with English question marks in verbatim text.</t>
+        </is>
+      </c>
+      <c r="F62" s="121" t="n"/>
+      <c r="G62" s="121" t="n"/>
+      <c r="H62" s="121" t="n"/>
+      <c r="I62" s="121" t="n"/>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="134" t="inlineStr">
+        <is>
+          <t>Pitch ↑↓</t>
+        </is>
+      </c>
+      <c r="B63" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"[↑↓]", text))</t>
+        </is>
+      </c>
+      <c r="C63" s="121" t="n"/>
+      <c r="D63" s="121" t="n"/>
+      <c r="E63" s="129" t="inlineStr">
+        <is>
+          <t>Unicode pitch arrows.</t>
+        </is>
+      </c>
+      <c r="F63" s="121" t="n"/>
+      <c r="G63" s="121" t="n"/>
+      <c r="H63" s="121" t="n"/>
+      <c r="I63" s="121" t="n"/>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="134" t="inlineStr">
+        <is>
+          <t>Lengthening ::</t>
+        </is>
+      </c>
+      <c r="B64" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r":{2,}", text))</t>
+        </is>
+      </c>
+      <c r="C64" s="121" t="n"/>
+      <c r="D64" s="121" t="n"/>
+      <c r="E64" s="129" t="inlineStr">
+        <is>
+          <t>2+ colons.</t>
+        </is>
+      </c>
+      <c r="F64" s="121" t="n"/>
+      <c r="G64" s="121" t="n"/>
+      <c r="H64" s="121" t="n"/>
+      <c r="I64" s="121" t="n"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="134" t="inlineStr">
+        <is>
+          <t>Emphasis __word__</t>
+        </is>
+      </c>
+      <c r="B65" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"__\S+__", text))</t>
+        </is>
+      </c>
+      <c r="C65" s="121" t="n"/>
+      <c r="D65" s="121" t="n"/>
+      <c r="E65" s="129" t="inlineStr">
+        <is>
+          <t>Double-underscore-wrapped token (\S+ = non-whitespace).</t>
+        </is>
+      </c>
+      <c r="F65" s="121" t="n"/>
+      <c r="G65" s="121" t="n"/>
+      <c r="H65" s="121" t="n"/>
+      <c r="I65" s="121" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="134" t="inlineStr">
+        <is>
+          <t>Cutoff word-</t>
+        </is>
+      </c>
+      <c r="B66" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\w+-(?=\s|$)", text, re.M))</t>
+        </is>
+      </c>
+      <c r="C66" s="121" t="n"/>
+      <c r="D66" s="121" t="n"/>
+      <c r="E66" s="129" t="inlineStr">
+        <is>
+          <t>Word followed by hyphen at end of word boundary — lookahead for whitespace or line end.</t>
+        </is>
+      </c>
+      <c r="F66" s="121" t="n"/>
+      <c r="G66" s="121" t="n"/>
+      <c r="H66" s="121" t="n"/>
+      <c r="I66" s="121" t="n"/>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="134" t="inlineStr">
+        <is>
+          <t>Loud CAPS</t>
+        </is>
+      </c>
+      <c r="B67" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\b[A-Z]{2,}\b", text))</t>
+        </is>
+      </c>
+      <c r="C67" s="121" t="n"/>
+      <c r="D67" s="121" t="n"/>
+      <c r="E67" s="129" t="inlineStr">
+        <is>
+          <t>2+ capital letters as a word.</t>
+        </is>
+      </c>
+      <c r="F67" s="121" t="n"/>
+      <c r="G67" s="121" t="n"/>
+      <c r="H67" s="121" t="n"/>
+      <c r="I67" s="121" t="n"/>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="134" t="inlineStr">
+        <is>
+          <t>Beat pause (.)</t>
+        </is>
+      </c>
+      <c r="B68" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\.{1,3}\)", text))</t>
+        </is>
+      </c>
+      <c r="C68" s="121" t="n"/>
+      <c r="D68" s="121" t="n"/>
+      <c r="E68" s="129" t="inlineStr">
+        <is>
+          <t>Parenthesised 1–3 dots (beat pauses).</t>
+        </is>
+      </c>
+      <c r="F68" s="121" t="n"/>
+      <c r="G68" s="121" t="n"/>
+      <c r="H68" s="121" t="n"/>
+      <c r="I68" s="121" t="n"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="134" t="inlineStr">
+        <is>
+          <t>Timed pause (n.n)</t>
+        </is>
+      </c>
+      <c r="B69" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\d+\.?\d*\)", text))</t>
+        </is>
+      </c>
+      <c r="C69" s="121" t="n"/>
+      <c r="D69" s="121" t="n"/>
+      <c r="E69" s="129" t="inlineStr">
+        <is>
+          <t>Parenthesised number in seconds.</t>
+        </is>
+      </c>
+      <c r="F69" s="121" t="n"/>
+      <c r="G69" s="121" t="n"/>
+      <c r="H69" s="121" t="n"/>
+      <c r="I69" s="121" t="n"/>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="134" t="inlineStr">
+        <is>
+          <t>Latching =</t>
+        </is>
+      </c>
+      <c r="B70" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"=", text))</t>
+        </is>
+      </c>
+      <c r="C70" s="121" t="n"/>
+      <c r="D70" s="121" t="n"/>
+      <c r="E70" s="129">
+        <f> signs.</f>
+        <v/>
+      </c>
+      <c r="F70" s="121" t="n"/>
+      <c r="G70" s="121" t="n"/>
+      <c r="H70" s="121" t="n"/>
+      <c r="I70" s="121" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="134" t="inlineStr">
+        <is>
+          <t>Overlap start [</t>
+        </is>
+      </c>
+      <c r="B71" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\[", text))</t>
+        </is>
+      </c>
+      <c r="C71" s="121" t="n"/>
+      <c r="D71" s="121" t="n"/>
+      <c r="E71" s="129" t="inlineStr">
+        <is>
+          <t>[ brackets.</t>
+        </is>
+      </c>
+      <c r="F71" s="121" t="n"/>
+      <c r="G71" s="121" t="n"/>
+      <c r="H71" s="121" t="n"/>
+      <c r="I71" s="121" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="134" t="inlineStr">
+        <is>
+          <t>Overlap end *</t>
+        </is>
+      </c>
+      <c r="B72" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\*", text))</t>
+        </is>
+      </c>
+      <c r="C72" s="121" t="n"/>
+      <c r="D72" s="121" t="n"/>
+      <c r="E72" s="129" t="inlineStr">
+        <is>
+          <t>* characters.</t>
+        </is>
+      </c>
+      <c r="F72" s="121" t="n"/>
+      <c r="G72" s="121" t="n"/>
+      <c r="H72" s="121" t="n"/>
+      <c r="I72" s="121" t="n"/>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="134" t="inlineStr">
+        <is>
+          <t>Voice quality {..}</t>
+        </is>
+      </c>
+      <c r="B73" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\{[A-Za-z ]+\}", text))</t>
+        </is>
+      </c>
+      <c r="C73" s="121" t="n"/>
+      <c r="D73" s="121" t="n"/>
+      <c r="E73" s="129" t="inlineStr">
+        <is>
+          <t>Curly-bracket voice quality annotations like {B} {piano}.</t>
+        </is>
+      </c>
+      <c r="F73" s="121" t="n"/>
+      <c r="G73" s="121" t="n"/>
+      <c r="H73" s="121" t="n"/>
+      <c r="I73" s="121" t="n"/>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="134" t="inlineStr">
+        <is>
+          <t>Intelligibility (xXx)</t>
+        </is>
+      </c>
+      <c r="B74" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\([xX]+\)", text))</t>
+        </is>
+      </c>
+      <c r="C74" s="121" t="n"/>
+      <c r="D74" s="121" t="n"/>
+      <c r="E74" s="129" t="inlineStr">
+        <is>
+          <t>Parenthesised x/X syllable patterns.</t>
+        </is>
+      </c>
+      <c r="F74" s="121" t="n"/>
+      <c r="G74" s="121" t="n"/>
+      <c r="H74" s="121" t="n"/>
+      <c r="I74" s="121" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="134" t="inlineStr">
+        <is>
+          <t>Non-verbal ((..))</t>
+        </is>
+      </c>
+      <c r="B75" s="123" t="inlineStr">
+        <is>
+          <t>len(re.findall(r"\(\(.*?\)\)", text))</t>
+        </is>
+      </c>
+      <c r="C75" s="121" t="n"/>
+      <c r="D75" s="121" t="n"/>
+      <c r="E75" s="129" t="inlineStr">
+        <is>
+          <t>Double-parenthesis non-verbal annotations.</t>
+        </is>
+      </c>
+      <c r="F75" s="121" t="n"/>
+      <c r="G75" s="121" t="n"/>
+      <c r="H75" s="121" t="n"/>
+      <c r="I75" s="121" t="n"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="119" t="inlineStr">
+        <is>
+          <t>STEP 5 — CV Calculation: Mean, Standard Deviation, Coefficient of Variation</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="135" t="inlineStr">
+        <is>
+          <t>CV (Coefficient of Variation) = Standard Deviation ÷ Mean, computed across the 5 models within one notation. Each model value is its average Total Markers across 4 clips. Higher CV = models differ more from each other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1">
+      <c r="A79" s="127" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B79" s="127" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C79" s="121" t="n"/>
+      <c r="D79" s="121" t="n"/>
+      <c r="E79" s="121" t="n"/>
+      <c r="F79" s="121" t="n"/>
+      <c r="G79" s="121" t="n"/>
+      <c r="H79" s="121" t="n"/>
+      <c r="I79" s="121" t="n"/>
+    </row>
+    <row r="80" ht="28" customHeight="1">
+      <c r="A80" s="136" t="inlineStr">
+        <is>
+          <t>Step 1 — Raw values</t>
+        </is>
+      </c>
+      <c r="B80" s="137" t="inlineStr">
+        <is>
+          <t>Read Total Markers for each of the 80 indexed files (5 models × 4 notations × 4 clips).</t>
+        </is>
+      </c>
+      <c r="C80" s="121" t="n"/>
+      <c r="D80" s="121" t="n"/>
+      <c r="E80" s="121" t="n"/>
+      <c r="F80" s="121" t="n"/>
+      <c r="G80" s="121" t="n"/>
+      <c r="H80" s="121" t="n"/>
+      <c r="I80" s="121" t="n"/>
+    </row>
+    <row r="81" ht="28" customHeight="1">
+      <c r="A81" s="136" t="inlineStr">
+        <is>
+          <t>Step 2 — Per-model mean</t>
+        </is>
+      </c>
+      <c r="B81" s="137" t="inlineStr">
+        <is>
+          <t>For each model, average its 4 clip scores → 5 values (one per model).
+  Example (Müller): Gemini Pro = (48+26+58+10)/4 = 35.5</t>
+        </is>
+      </c>
+      <c r="C81" s="121" t="n"/>
+      <c r="D81" s="121" t="n"/>
+      <c r="E81" s="121" t="n"/>
+      <c r="F81" s="121" t="n"/>
+      <c r="G81" s="121" t="n"/>
+      <c r="H81" s="121" t="n"/>
+      <c r="I81" s="121" t="n"/>
+    </row>
+    <row r="82" ht="28" customHeight="1">
+      <c r="A82" s="136" t="inlineStr">
+        <is>
+          <t>Step 3 — Grand mean (μ)</t>
+        </is>
+      </c>
+      <c r="B82" s="137" t="inlineStr">
+        <is>
+          <t>Average of the 5 model-means.  Formula: μ = Σ(model_mean) / 5</t>
+        </is>
+      </c>
+      <c r="C82" s="121" t="n"/>
+      <c r="D82" s="121" t="n"/>
+      <c r="E82" s="121" t="n"/>
+      <c r="F82" s="121" t="n"/>
+      <c r="G82" s="121" t="n"/>
+      <c r="H82" s="121" t="n"/>
+      <c r="I82" s="121" t="n"/>
+    </row>
+    <row r="83" ht="28" customHeight="1">
+      <c r="A83" s="136" t="inlineStr">
+        <is>
+          <t>Step 4 — Std deviation (σ)</t>
+        </is>
+      </c>
+      <c r="B83" s="137" t="inlineStr">
+        <is>
+          <t>σ = √[ Σ(model_mean − μ)² / (n−1) ]   (sample standard deviation, pandas ddof=1)</t>
+        </is>
+      </c>
+      <c r="C83" s="121" t="n"/>
+      <c r="D83" s="121" t="n"/>
+      <c r="E83" s="121" t="n"/>
+      <c r="F83" s="121" t="n"/>
+      <c r="G83" s="121" t="n"/>
+      <c r="H83" s="121" t="n"/>
+      <c r="I83" s="121" t="n"/>
+    </row>
+    <row r="84" ht="28" customHeight="1">
+      <c r="A84" s="136" t="inlineStr">
+        <is>
+          <t>Step 5 — CV</t>
+        </is>
+      </c>
+      <c r="B84" s="137" t="inlineStr">
+        <is>
+          <t>CV = σ / μ   Dimensionless — allows fair comparison between notations that have different absolute marker counts.</t>
+        </is>
+      </c>
+      <c r="C84" s="121" t="n"/>
+      <c r="D84" s="121" t="n"/>
+      <c r="E84" s="121" t="n"/>
+      <c r="F84" s="121" t="n"/>
+      <c r="G84" s="121" t="n"/>
+      <c r="H84" s="121" t="n"/>
+      <c r="I84" s="121" t="n"/>
+    </row>
+    <row r="85" ht="28" customHeight="1">
+      <c r="A85" s="136" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="B85" s="137" t="inlineStr">
+        <is>
+          <t>CV &lt; 0.20 → low (models barely differ)  |  CV 0.40–0.60 → high  |  CV &gt; 0.60 → very high (outlier model present)</t>
+        </is>
+      </c>
+      <c r="C85" s="121" t="n"/>
+      <c r="D85" s="121" t="n"/>
+      <c r="E85" s="121" t="n"/>
+      <c r="F85" s="121" t="n"/>
+      <c r="G85" s="121" t="n"/>
+      <c r="H85" s="121" t="n"/>
+      <c r="I85" s="121" t="n"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="138" t="inlineStr">
+        <is>
+          <t>RAW DATA MATRICES — Total Markers per Model × Clip, with Mean / Deviation from Grand Mean / CV</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Jefferson (CA)   (CV = 0.549)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="28" customHeight="1">
+      <c r="A90" s="127" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B90" s="127" t="inlineStr">
+        <is>
+          <t>Apollo13</t>
+        </is>
+      </c>
+      <c r="C90" s="127" t="inlineStr">
+        <is>
+          <t>PaperChain</t>
+        </is>
+      </c>
+      <c r="D90" s="127" t="inlineStr">
+        <is>
+          <t>Primer</t>
+        </is>
+      </c>
+      <c r="E90" s="127" t="inlineStr">
+        <is>
+          <t>Meyerowitz</t>
+        </is>
+      </c>
+      <c r="F90" s="139" t="inlineStr">
+        <is>
+          <t>Mean
+(4 clips)</t>
+        </is>
+      </c>
+      <c r="G90" s="139" t="inlineStr">
+        <is>
+          <t>Dev from
+grand mean</t>
+        </is>
+      </c>
+      <c r="H90" s="131" t="inlineStr">
+        <is>
+          <t>CV
+(σ/μ)</t>
+        </is>
+      </c>
+      <c r="I90" s="140" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="17" customHeight="1">
+      <c r="A91" s="141" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="B91" s="142" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C91" s="142" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D91" s="142" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E91" s="142" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F91" s="143" t="n">
+        <v>23</v>
+      </c>
+      <c r="G91" s="144" t="inlineStr">
+        <is>
+          <t>+6.8</t>
+        </is>
+      </c>
+      <c r="H91" s="121" t="inlineStr"/>
+      <c r="I91" s="145" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="17" customHeight="1">
+      <c r="A92" s="141" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Flash</t>
+        </is>
+      </c>
+      <c r="B92" s="142" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C92" s="142" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D92" s="142" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E92" s="142" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F92" s="143" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G92" s="146" t="inlineStr">
+        <is>
+          <t>-2.8</t>
+        </is>
+      </c>
+      <c r="H92" s="121" t="inlineStr"/>
+      <c r="I92" s="145" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="17" customHeight="1">
+      <c r="A93" s="141" t="inlineStr">
+        <is>
+          <t>GPT-audio</t>
+        </is>
+      </c>
+      <c r="B93" s="142" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C93" s="142" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D93" s="142" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E93" s="142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F93" s="143" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="G93" s="144" t="inlineStr">
+        <is>
+          <t>+5.2</t>
+        </is>
+      </c>
+      <c r="H93" s="121" t="inlineStr"/>
+      <c r="I93" s="145" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="17" customHeight="1">
+      <c r="A94" s="141" t="inlineStr">
+        <is>
+          <t>GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="B94" s="142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C94" s="142" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D94" s="142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E94" s="142" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F94" s="143" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G94" s="146" t="inlineStr">
+        <is>
+          <t>-14.5</t>
+        </is>
+      </c>
+      <c r="H94" s="121" t="inlineStr"/>
+      <c r="I94" s="145" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="17" customHeight="1">
+      <c r="A95" s="141" t="inlineStr">
+        <is>
+          <t>WhisperX medium</t>
+        </is>
+      </c>
+      <c r="B95" s="142" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C95" s="142" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D95" s="142" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E95" s="142" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F95" s="143" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="G95" s="144" t="inlineStr">
+        <is>
+          <t>+5.2</t>
+        </is>
+      </c>
+      <c r="H95" s="121" t="inlineStr"/>
+      <c r="I95" s="145" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="147" t="inlineStr">
+        <is>
+          <t>Grand mean / σ / CV →</t>
+        </is>
+      </c>
+      <c r="B96" s="148" t="n"/>
+      <c r="C96" s="148" t="n"/>
+      <c r="D96" s="148" t="n"/>
+      <c r="E96" s="148" t="n"/>
+      <c r="F96" s="149" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="G96" s="149" t="inlineStr">
+        <is>
+          <t>σ = 8.92</t>
+        </is>
+      </c>
+      <c r="H96" s="150" t="inlineStr">
+        <is>
+          <t>0.549
+MED</t>
+        </is>
+      </c>
+      <c r="I96" s="151" t="inlineStr"/>
+    </row>
+    <row r="97" ht="16" customHeight="1">
+      <c r="A97" s="152" t="inlineStr">
+        <is>
+          <t>μ=16.25  σ=8.92  CV=σ/μ=0.549  |  Dev from mean column shows each model's distance from μ</t>
+        </is>
+      </c>
+      <c r="B97" s="121" t="n"/>
+      <c r="C97" s="121" t="n"/>
+      <c r="D97" s="121" t="n"/>
+      <c r="E97" s="121" t="n"/>
+      <c r="F97" s="121" t="n"/>
+      <c r="G97" s="121" t="n"/>
+      <c r="H97" s="121" t="n"/>
+      <c r="I97" s="121" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Poland (2001)   (CV = 0.540)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="120" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B100" s="120" t="inlineStr">
+        <is>
+          <t>Apollo13</t>
+        </is>
+      </c>
+      <c r="C100" s="120" t="inlineStr">
+        <is>
+          <t>PaperChain</t>
+        </is>
+      </c>
+      <c r="D100" s="120" t="inlineStr">
+        <is>
+          <t>Primer</t>
+        </is>
+      </c>
+      <c r="E100" s="120" t="inlineStr">
+        <is>
+          <t>Meyerowitz</t>
+        </is>
+      </c>
+      <c r="F100" s="139" t="inlineStr">
+        <is>
+          <t>Mean
+(4 clips)</t>
+        </is>
+      </c>
+      <c r="G100" s="139" t="inlineStr">
+        <is>
+          <t>Dev from
+grand mean</t>
+        </is>
+      </c>
+      <c r="H100" s="131" t="inlineStr">
+        <is>
+          <t>CV
+(σ/μ)</t>
+        </is>
+      </c>
+      <c r="I100" s="140" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="17" customHeight="1">
+      <c r="A101" s="153" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="B101" s="154" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C101" s="154" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D101" s="154" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E101" s="154" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F101" s="155" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G101" s="156" t="inlineStr">
+        <is>
+          <t>-1.1</t>
+        </is>
+      </c>
+      <c r="H101" s="121" t="inlineStr"/>
+      <c r="I101" s="157" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="17" customHeight="1">
+      <c r="A102" s="153" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Flash</t>
+        </is>
+      </c>
+      <c r="B102" s="154" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C102" s="154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D102" s="154" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E102" s="154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F102" s="155" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="G102" s="156" t="inlineStr">
+        <is>
+          <t>+0.4</t>
+        </is>
+      </c>
+      <c r="H102" s="121" t="inlineStr"/>
+      <c r="I102" s="157" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="17" customHeight="1">
+      <c r="A103" s="153" t="inlineStr">
+        <is>
+          <t>GPT-audio</t>
+        </is>
+      </c>
+      <c r="B103" s="154" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="C103" s="154" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D103" s="154" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E103" s="154" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F103" s="155" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G103" s="158" t="inlineStr">
+        <is>
+          <t>+11.9</t>
+        </is>
+      </c>
+      <c r="H103" s="121" t="inlineStr"/>
+      <c r="I103" s="157" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="17" customHeight="1">
+      <c r="A104" s="153" t="inlineStr">
+        <is>
+          <t>GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="B104" s="154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C104" s="154" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D104" s="154" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E104" s="154" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F104" s="155" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G104" s="159" t="inlineStr">
+        <is>
+          <t>-14.1</t>
+        </is>
+      </c>
+      <c r="H104" s="121" t="inlineStr"/>
+      <c r="I104" s="157" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="17" customHeight="1">
+      <c r="A105" s="153" t="inlineStr">
+        <is>
+          <t>WhisperX medium</t>
+        </is>
+      </c>
+      <c r="B105" s="154" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C105" s="154" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D105" s="154" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E105" s="154" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F105" s="155" t="n">
+        <v>20</v>
+      </c>
+      <c r="G105" s="158" t="inlineStr">
+        <is>
+          <t>+2.7</t>
+        </is>
+      </c>
+      <c r="H105" s="121" t="inlineStr"/>
+      <c r="I105" s="157" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="147" t="inlineStr">
+        <is>
+          <t>Grand mean / σ / CV →</t>
+        </is>
+      </c>
+      <c r="B106" s="148" t="n"/>
+      <c r="C106" s="148" t="n"/>
+      <c r="D106" s="148" t="n"/>
+      <c r="E106" s="148" t="n"/>
+      <c r="F106" s="149" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G106" s="149" t="inlineStr">
+        <is>
+          <t>σ = 9.34</t>
+        </is>
+      </c>
+      <c r="H106" s="150" t="inlineStr">
+        <is>
+          <t>0.54
+MED</t>
+        </is>
+      </c>
+      <c r="I106" s="151" t="inlineStr"/>
+    </row>
+    <row r="107" ht="16" customHeight="1">
+      <c r="A107" s="152" t="inlineStr">
+        <is>
+          <t>μ=17.3  σ=9.34  CV=σ/μ=0.54  |  Dev from mean column shows each model's distance from μ</t>
+        </is>
+      </c>
+      <c r="B107" s="121" t="n"/>
+      <c r="C107" s="121" t="n"/>
+      <c r="D107" s="121" t="n"/>
+      <c r="E107" s="121" t="n"/>
+      <c r="F107" s="121" t="n"/>
+      <c r="G107" s="121" t="n"/>
+      <c r="H107" s="121" t="n"/>
+      <c r="I107" s="121" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Braun &amp; Clarke (2021)   (CV = 0.409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="28" customHeight="1">
+      <c r="A110" s="131" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B110" s="131" t="inlineStr">
+        <is>
+          <t>Apollo13</t>
+        </is>
+      </c>
+      <c r="C110" s="131" t="inlineStr">
+        <is>
+          <t>PaperChain</t>
+        </is>
+      </c>
+      <c r="D110" s="131" t="inlineStr">
+        <is>
+          <t>Primer</t>
+        </is>
+      </c>
+      <c r="E110" s="131" t="inlineStr">
+        <is>
+          <t>Meyerowitz</t>
+        </is>
+      </c>
+      <c r="F110" s="139" t="inlineStr">
+        <is>
+          <t>Mean
+(4 clips)</t>
+        </is>
+      </c>
+      <c r="G110" s="139" t="inlineStr">
+        <is>
+          <t>Dev from
+grand mean</t>
+        </is>
+      </c>
+      <c r="H110" s="131" t="inlineStr">
+        <is>
+          <t>CV
+(σ/μ)</t>
+        </is>
+      </c>
+      <c r="I110" s="140" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="17" customHeight="1">
+      <c r="A111" s="160" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="B111" s="161" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C111" s="161" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D111" s="161" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E111" s="161" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F111" s="162" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G111" s="163" t="inlineStr">
+        <is>
+          <t>+1.6</t>
+        </is>
+      </c>
+      <c r="H111" s="121" t="inlineStr"/>
+      <c r="I111" s="164" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="17" customHeight="1">
+      <c r="A112" s="160" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Flash</t>
+        </is>
+      </c>
+      <c r="B112" s="161" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C112" s="161" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D112" s="161" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E112" s="161" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F112" s="162" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G112" s="163" t="inlineStr">
+        <is>
+          <t>-0.2</t>
+        </is>
+      </c>
+      <c r="H112" s="121" t="inlineStr"/>
+      <c r="I112" s="164" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="17" customHeight="1">
+      <c r="A113" s="160" t="inlineStr">
+        <is>
+          <t>GPT-audio</t>
+        </is>
+      </c>
+      <c r="B113" s="161" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C113" s="161" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D113" s="161" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E113" s="161" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F113" s="162" t="n">
+        <v>17</v>
+      </c>
+      <c r="G113" s="165" t="inlineStr">
+        <is>
+          <t>+6.1</t>
+        </is>
+      </c>
+      <c r="H113" s="121" t="inlineStr"/>
+      <c r="I113" s="164" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="17" customHeight="1">
+      <c r="A114" s="160" t="inlineStr">
+        <is>
+          <t>GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="B114" s="161" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C114" s="161" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D114" s="161" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E114" s="161" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F114" s="162" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G114" s="166" t="inlineStr">
+        <is>
+          <t>-6.2</t>
+        </is>
+      </c>
+      <c r="H114" s="121" t="inlineStr"/>
+      <c r="I114" s="164" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="17" customHeight="1">
+      <c r="A115" s="160" t="inlineStr">
+        <is>
+          <t>WhisperX medium</t>
+        </is>
+      </c>
+      <c r="B115" s="161" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C115" s="161" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D115" s="161" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E115" s="161" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F115" s="162" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G115" s="163" t="inlineStr">
+        <is>
+          <t>-1.4</t>
+        </is>
+      </c>
+      <c r="H115" s="121" t="inlineStr"/>
+      <c r="I115" s="164" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="147" t="inlineStr">
+        <is>
+          <t>Grand mean / σ / CV →</t>
+        </is>
+      </c>
+      <c r="B116" s="148" t="n"/>
+      <c r="C116" s="148" t="n"/>
+      <c r="D116" s="148" t="n"/>
+      <c r="E116" s="148" t="n"/>
+      <c r="F116" s="149" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G116" s="149" t="inlineStr">
+        <is>
+          <t>σ = 4.46</t>
+        </is>
+      </c>
+      <c r="H116" s="150" t="inlineStr">
+        <is>
+          <t>0.409
+MED</t>
+        </is>
+      </c>
+      <c r="I116" s="151" t="inlineStr"/>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="152" t="inlineStr">
+        <is>
+          <t>μ=10.9  σ=4.46  CV=σ/μ=0.409  |  Dev from mean column shows each model's distance from μ</t>
+        </is>
+      </c>
+      <c r="B117" s="121" t="n"/>
+      <c r="C117" s="121" t="n"/>
+      <c r="D117" s="121" t="n"/>
+      <c r="E117" s="121" t="n"/>
+      <c r="F117" s="121" t="n"/>
+      <c r="G117" s="121" t="n"/>
+      <c r="H117" s="121" t="n"/>
+      <c r="I117" s="121" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Müller &amp; Guendouzi (2005)   (CV = 0.614  ← HIGHEST DISCRIMINATION ★)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="28" customHeight="1">
+      <c r="A120" s="133" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B120" s="133" t="inlineStr">
+        <is>
+          <t>Apollo13</t>
+        </is>
+      </c>
+      <c r="C120" s="133" t="inlineStr">
+        <is>
+          <t>PaperChain</t>
+        </is>
+      </c>
+      <c r="D120" s="133" t="inlineStr">
+        <is>
+          <t>Primer</t>
+        </is>
+      </c>
+      <c r="E120" s="133" t="inlineStr">
+        <is>
+          <t>Meyerowitz</t>
+        </is>
+      </c>
+      <c r="F120" s="139" t="inlineStr">
+        <is>
+          <t>Mean
+(4 clips)</t>
+        </is>
+      </c>
+      <c r="G120" s="139" t="inlineStr">
+        <is>
+          <t>Dev from
+grand mean</t>
+        </is>
+      </c>
+      <c r="H120" s="131" t="inlineStr">
+        <is>
+          <t>CV
+(σ/μ)</t>
+        </is>
+      </c>
+      <c r="I120" s="140" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="17" customHeight="1">
+      <c r="A121" s="168" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="B121" s="169" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C121" s="169" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D121" s="169" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E121" s="169" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F121" s="170" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="G121" s="171" t="inlineStr">
+        <is>
+          <t>+3.6</t>
+        </is>
+      </c>
+      <c r="H121" s="121" t="inlineStr"/>
+      <c r="I121" s="172" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="17" customHeight="1">
+      <c r="A122" s="168" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Flash</t>
+        </is>
+      </c>
+      <c r="B122" s="169" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C122" s="169" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D122" s="169" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E122" s="169" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F122" s="170" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G122" s="173" t="inlineStr">
+        <is>
+          <t>-13.1</t>
+        </is>
+      </c>
+      <c r="H122" s="121" t="inlineStr"/>
+      <c r="I122" s="172" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="17" customHeight="1">
+      <c r="A123" s="168" t="inlineStr">
+        <is>
+          <t>GPT-audio</t>
+        </is>
+      </c>
+      <c r="B123" s="169" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="C123" s="169" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D123" s="169" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E123" s="169" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="F123" s="170" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="G123" s="171" t="inlineStr">
+        <is>
+          <t>+30.9</t>
+        </is>
+      </c>
+      <c r="H123" s="121" t="inlineStr"/>
+      <c r="I123" s="172" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="17" customHeight="1">
+      <c r="A124" s="168" t="inlineStr">
+        <is>
+          <t>GPT-audio Mini</t>
+        </is>
+      </c>
+      <c r="B124" s="169" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C124" s="169" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D124" s="169" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E124" s="169" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F124" s="170" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G124" s="173" t="inlineStr">
+        <is>
+          <t>-19.1</t>
+        </is>
+      </c>
+      <c r="H124" s="121" t="inlineStr"/>
+      <c r="I124" s="172" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="17" customHeight="1">
+      <c r="A125" s="168" t="inlineStr">
+        <is>
+          <t>WhisperX medium</t>
+        </is>
+      </c>
+      <c r="B125" s="169" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C125" s="169" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D125" s="169" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E125" s="169" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F125" s="170" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="G125" s="173" t="inlineStr">
+        <is>
+          <t>-2.1</t>
+        </is>
+      </c>
+      <c r="H125" s="121" t="inlineStr"/>
+      <c r="I125" s="172" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="147" t="inlineStr">
+        <is>
+          <t>Grand mean / σ / CV →</t>
+        </is>
+      </c>
+      <c r="B126" s="148" t="n"/>
+      <c r="C126" s="148" t="n"/>
+      <c r="D126" s="148" t="n"/>
+      <c r="E126" s="148" t="n"/>
+      <c r="F126" s="149" t="n">
+        <v>31.65</v>
+      </c>
+      <c r="G126" s="149" t="inlineStr">
+        <is>
+          <t>σ = 19.42</t>
+        </is>
+      </c>
+      <c r="H126" s="150" t="inlineStr">
+        <is>
+          <t>0.614
+HIGH ★</t>
+        </is>
+      </c>
+      <c r="I126" s="151" t="inlineStr"/>
+    </row>
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="152" t="inlineStr">
+        <is>
+          <t>μ=31.65  σ=19.42  CV=σ/μ=0.614  |  Dev from mean column shows each model's distance from μ</t>
+        </is>
+      </c>
+      <c r="B127" s="121" t="n"/>
+      <c r="C127" s="121" t="n"/>
+      <c r="D127" s="121" t="n"/>
+      <c r="E127" s="121" t="n"/>
+      <c r="F127" s="121" t="n"/>
+      <c r="G127" s="121" t="n"/>
+      <c r="H127" s="121" t="n"/>
+      <c r="I127" s="121" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="143">
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="E68:I68"/>
+    <mergeCell ref="A99:I99"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E55:I55"/>
+    <mergeCell ref="E52:I52"/>
+    <mergeCell ref="E67:I67"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="A109:I109"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="A117:I117"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="B83:I83"/>
+    <mergeCell ref="E7:I7"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B85:I85"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A89:I89"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="E44:I44"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="E69:I69"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E46:I46"/>
+    <mergeCell ref="B75:D75"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="E61:I61"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E70:I70"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E72:I72"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E41:I41"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E47:I47"/>
+    <mergeCell ref="A78:I78"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E56:I56"/>
+    <mergeCell ref="E43:I43"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E8:I8"/>
+    <mergeCell ref="E53:I53"/>
+    <mergeCell ref="E35:I35"/>
+    <mergeCell ref="E19:I19"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E9:I9"/>
+    <mergeCell ref="E74:I74"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B79:I79"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="E71:I71"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E64:I64"/>
+    <mergeCell ref="E73:I73"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="E63:I63"/>
+    <mergeCell ref="A97:I97"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E65:I65"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A127:I127"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B84:I84"/>
+    <mergeCell ref="A107:I107"/>
+    <mergeCell ref="A60:I60"/>
+    <mergeCell ref="B71:D71"/>
+    <mergeCell ref="A88:I88"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E66:I66"/>
+    <mergeCell ref="E75:I75"/>
+    <mergeCell ref="B80:I80"/>
+    <mergeCell ref="E22:I22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>